<commit_message>
addition of accidents model to edgelist
</commit_message>
<xml_diff>
--- a/OSW Model Edgelists_v2.xlsx
+++ b/OSW Model Edgelists_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://007gc-my.sharepoint.com/personal/cody_dey_ec_gc_ca/Documents/Desktop/OSW Network Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://007gc.sharepoint.com/sites/msteams_f728f5/Shared Documents/General/Science Advice/In Progress Science Advice/OSW Aerofauna PoE/OSW-Network-Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="357" documentId="8_{4783B985-3D31-4373-BA0E-4DD94F8BE2BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AF7CE08-4DA7-4384-B235-B541CD6F9351}"/>
+  <xr:revisionPtr revIDLastSave="430" documentId="8_{4783B985-3D31-4373-BA0E-4DD94F8BE2BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BD16C97-1D2A-4954-9EE2-5201F95EB52C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{DB453CEF-A2F4-4F96-A3F5-4955188A497E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{DB453CEF-A2F4-4F96-A3F5-4955188A497E}"/>
   </bookViews>
   <sheets>
     <sheet name="Site Survey" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Routine Maintenance" sheetId="5" r:id="rId5"/>
     <sheet name="Full Removal" sheetId="6" r:id="rId6"/>
     <sheet name="Partial Removal" sheetId="7" r:id="rId7"/>
+    <sheet name="Accidents" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="94">
   <si>
     <t>Node Source</t>
   </si>
@@ -273,6 +274,60 @@
   </si>
   <si>
     <t>Habitat Loss_[Effect]</t>
+  </si>
+  <si>
+    <t>Chemical Hazard Introduction</t>
+  </si>
+  <si>
+    <t>Physical Hazard Introduction</t>
+  </si>
+  <si>
+    <t>Invasive Species Introduction</t>
+  </si>
+  <si>
+    <t>Oil Coating Plumage</t>
+  </si>
+  <si>
+    <t>Ingestion of Hazardous Substances</t>
+  </si>
+  <si>
+    <t>Lower Habitat Quality</t>
+  </si>
+  <si>
+    <t>Entanglement</t>
+  </si>
+  <si>
+    <t>Reduced Buoyancy</t>
+  </si>
+  <si>
+    <t>Reduced Thermal Regulation</t>
+  </si>
+  <si>
+    <t>Lower Prey Abundance</t>
+  </si>
+  <si>
+    <t>Increased Energy Cost</t>
+  </si>
+  <si>
+    <t>A_PH_Entanglement</t>
+  </si>
+  <si>
+    <t>A_CH_OilSpill</t>
+  </si>
+  <si>
+    <t>A_CH_Spill</t>
+  </si>
+  <si>
+    <t>A_CH_Spill, A_CH_Foundation, A_CH_Leach</t>
+  </si>
+  <si>
+    <t>A_PH_Debris</t>
+  </si>
+  <si>
+    <t>A_PH_Mechfail</t>
+  </si>
+  <si>
+    <t>A_IS_Forage</t>
   </si>
 </sst>
 </file>
@@ -3008,7 +3063,345 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F67AC817-86DF-460F-88BA-EFF3B0F6050E}">
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="2" max="2" width="33" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cc76eb8-63c4-49b5-af97-aa46e95f4cee">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="66572b97-5d1e-4594-b393-c33e0c30744c" xsi:nil="true"/>
+    <ProtectionClassification xmlns="5cc76eb8-63c4-49b5-af97-aa46e95f4cee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002A627B0EA5E1E043BA33477F76A4A51B" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9f6b5fe63d52f73b6f6710187ef903d1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5cc76eb8-63c4-49b5-af97-aa46e95f4cee" xmlns:ns3="66572b97-5d1e-4594-b393-c33e0c30744c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7563e552e9b75cc09e606806e9844d8" ns2:_="" ns3:_="">
     <xsd:import namespace="5cc76eb8-63c4-49b5-af97-aa46e95f4cee"/>
@@ -3253,35 +3646,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cc76eb8-63c4-49b5-af97-aa46e95f4cee">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="66572b97-5d1e-4594-b393-c33e0c30744c" xsi:nil="true"/>
-    <ProtectionClassification xmlns="5cc76eb8-63c4-49b5-af97-aa46e95f4cee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{139DA207-5799-4B09-9F6D-DC708A6D1AF5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D7B5F6B-E625-4B68-9B95-B9D75EE8AD03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5cc76eb8-63c4-49b5-af97-aa46e95f4cee"/>
+    <ds:schemaRef ds:uri="66572b97-5d1e-4594-b393-c33e0c30744c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A75D0B8-ACA3-468E-9239-FDD88B28D33A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A75D0B8-ACA3-468E-9239-FDD88B28D33A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D7B5F6B-E625-4B68-9B95-B9D75EE8AD03}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{139DA207-5799-4B09-9F6D-DC708A6D1AF5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5cc76eb8-63c4-49b5-af97-aa46e95f4cee"/>
+    <ds:schemaRef ds:uri="66572b97-5d1e-4594-b393-c33e0c30744c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>